<commit_message>
Fix: permissions marked as partial (UI only, not enforced)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WikiLive шаблон фич.xlsx
+++ b/WikiLive шаблон фич.xlsx
@@ -406,7 +406,7 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Интеграция с MWS Tables через API</t>
         </is>
@@ -431,7 +431,7 @@
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Создание и редактирование вики-страницы в сценарии MWS Tables</t>
         </is>
@@ -456,7 +456,7 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Вставка существующей таблицы MWS Tables в тело страницы (встраивание, не только ссылка)</t>
         </is>
@@ -481,7 +481,7 @@
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Автосохранение при редактировании и восстановление после перезагрузки / возврата (в т.ч. локальный кеш)</t>
         </is>
@@ -506,7 +506,7 @@
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Slash-menu для быстрого добавления блоков</t>
         </is>
@@ -531,7 +531,7 @@
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Горячие клавиши для slash-menu / ключевых команд редактора (перечень в README)</t>
         </is>
@@ -556,7 +556,7 @@
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Ссылки на другие страницы и обратные ссылки (backlinks)</t>
         </is>
@@ -581,7 +581,7 @@
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Совместная работа над документом (проверяемый сценарий)</t>
         </is>
@@ -606,7 +606,7 @@
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Редактор на open-source основе, permissive лицензия (MIT-like)</t>
         </is>
@@ -631,7 +631,7 @@
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Таблица на странице как «живой» объект (синхронизация с MWS Tables)</t>
         </is>
@@ -656,7 +656,7 @@
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Комментирование</t>
         </is>
@@ -681,7 +681,7 @@
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Версионирование / история правок / отдельные черновики</t>
         </is>
@@ -706,7 +706,7 @@
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>AI-подсказки или генерация блоков</t>
         </is>
@@ -731,7 +731,7 @@
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Граф связей между страницами</t>
         </is>
@@ -756,7 +756,7 @@
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Плагины / расширяемость редактора</t>
         </is>
@@ -781,7 +781,7 @@
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Встраивание внешних элементов (виджеты, превью и т.д.)</t>
         </is>
@@ -806,7 +806,7 @@
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Соответствие Design Kit</t>
         </is>
@@ -831,7 +831,7 @@
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>0 строк бэкенда написано</t>
         </is>
@@ -853,20 +853,20 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="0" t="inlineStr">
         <is>
           <t>E2E-шифрование данных</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>дополнительная</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -878,20 +878,20 @@
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="5">
-      <c r="A21" t="n">
+      <c r="A21" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="0" t="inlineStr">
         <is>
           <t>Proof of Work защита от флуда</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>дополнительная</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -903,20 +903,20 @@
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="5">
-      <c r="A22" t="n">
+      <c r="A22" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="0" t="inlineStr">
         <is>
           <t>Регистрация за 0 кликов</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>дополнительная</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -928,20 +928,20 @@
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="5">
-      <c r="A23" t="n">
+      <c r="A23" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="0" t="inlineStr">
         <is>
           <t>CRDT real-time синхронизация без конфликтов</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>дополнительная</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -953,20 +953,20 @@
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="5">
-      <c r="A24" t="n">
+      <c r="A24" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="0" t="inlineStr">
         <is>
           <t>Offline First — полноценная работа без интернета</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>дополнительная</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -978,20 +978,20 @@
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="5">
-      <c r="A25" t="n">
+      <c r="A25" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="0" t="inlineStr">
         <is>
           <t>Graceful degradation — устойчивость к потере сети</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>дополнительная</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -1003,45 +1003,45 @@
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="5">
-      <c r="A26" t="n">
+      <c r="A26" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="0" t="inlineStr">
         <is>
           <t>Права доступа (owner / editor / viewer)</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>дополнительная</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Да</t>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>Частично</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Ролевая модель на уровне Giper Baza Land: Owner (полный доступ + управление правами), Editor (редактирование), Viewer (только чтение). UI адаптируется: скрываются кнопки, блокируется ввод.</t>
+          <t>Визуальная часть готова: UI панели прав, отображение ролей (Owner/Editor/Viewer), скрытие кнопок редактирования для Viewer. Логика Giper Baza land.pass_rank() подключена, но реальное ограничение записи на уровне CRDT пока не проверено в продакшне.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="5">
-      <c r="A27" t="n">
+      <c r="A27" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="0" t="inlineStr">
         <is>
           <t>Адаптивность на все размеры экранов</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>дополнительная</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -1053,20 +1053,20 @@
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="5">
-      <c r="A28" t="n">
+      <c r="A28" s="0" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="0" t="inlineStr">
         <is>
           <t>Билды под все ОС (Web + Desktop)</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t>дополнительная</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -1078,20 +1078,20 @@
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="5">
-      <c r="A29" t="n">
+      <c r="A29" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="0" t="inlineStr">
         <is>
           <t>Web Component — приложение как встраиваемый компонент</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>дополнительная</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -1103,20 +1103,20 @@
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="5">
-      <c r="A30" t="n">
+      <c r="A30" s="0" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="0" t="inlineStr">
         <is>
           <t>Локализация (RU + EN, расширяемая)</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>дополнительная</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="0" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -1128,20 +1128,20 @@
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="5">
-      <c r="A31" t="n">
+      <c r="A31" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="0" t="inlineStr">
         <is>
           <t>Pull-реактивность без Virtual DOM</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>дополнительная</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
@@ -1153,20 +1153,20 @@
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="5">
-      <c r="A32" t="n">
+      <c r="A32" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="0" t="inlineStr">
         <is>
           <t>Светлая и тёмная тема из коробки</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>дополнительная</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t>Да</t>
         </is>

</xml_diff>

<commit_message>
Simplify feature descriptions, reorder: Web Component higher
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WikiLive шаблон фич.xlsx
+++ b/WikiLive шаблон фич.xlsx
@@ -423,7 +423,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>$bog_wiki_model — полноценный API-клиент MWS Fusion API v1. 8 эндпоинтов: GET spaces, nodes, views, records, fields + POST/PATCH/DELETE records. Авторизация Bearer token. Запросы через CORS-прокси. Реактивный кеш через @$mol_mem_key с ревизиями.</t>
+          <t>API-клиент MWS Fusion API v1. 8 эндпоинтов (CRUD records, views, fields, spaces). Bearer token. CORS-прокси.</t>
         </is>
       </c>
     </row>
@@ -448,7 +448,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>WYSIWYG-редактор на $mol (contenteditable). Блочная структура: параграфы, заголовки H1–H6, списки, цитаты, код, изображения, embed. Giper Baza CRDT хранит каждую страницу как отдельный Land с типизированными Pawn-блоками. Реестры и страницы с сайдбаром.</t>
+          <t>WYSIWYG на $mol, contenteditable, блочная структура. Хранение в Giper Baza CRDT.</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Slash-menu → «MWS Table» → ввод dstId + viewId → живая таблица рендерится inline как $mol-компонент прямо в теле страницы. Plugin Registry с render() callback. WeakMap-кеш компонентов. contentEditable=false для блока таблицы.</t>
+          <t>Slash-menu → MWS Table → dstId → живая таблица inline в теле страницы. Plugin Registry.</t>
         </is>
       </c>
     </row>
@@ -498,7 +498,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Giper Baza CRDT — автосохранение каждого нажатия в реальном времени. Данные в IndexedDB на клиенте. При перезагрузке — мгновенное восстановление из локального кеша. 0 строк бэкенда — бэкенд не нужен.</t>
+          <t>Giper Baza CRDT — автосохранение в реальном времени, IndexedDB. 0 строк бэкенда.</t>
         </is>
       </c>
     </row>
@@ -523,7 +523,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>«/» в пустом блоке открывает slash-menu со всеми доступными типами блоков: параграф, заголовки H1–H6, список, цитата, код, изображение, embed, MWS Table, AI. Реализовано через $bog_wysiwyg_plugin_registry.</t>
+          <t>«/» в блоке → меню всех типов блоков. $bog_wysiwyg_plugin_registry.</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Enter — новый блок, Backspace в пустом — удалить блок, Tab/Shift+Tab — изменить уровень. Markdown-шорткаты: # → H1, ## → H2, &gt; → цитата, ``` → код, - → список. Drag &amp; drop для перетаскивания блоков.</t>
+          <t>Enter, Backspace, Tab/Shift+Tab, Markdown-шорткаты (#, &gt;, ```, -). Drag &amp; drop блоков.</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Wikilinks [[page]] для ссылок между страницами. Backlinks — автоматический поиск обратных ссылок по HTML-контенту всех блоков всех страниц. all_pages_info() собирает данные для поиска.</t>
+          <t>Wikilinks [[page]], автоматические backlinks по всем страницам.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Giper Baza CRDT — real-time синхронизация между всеми клиентами без конфликтов. Каждая страница — отдельный Land. Несколько пользователей одновременно редактируют один документ, изменения мержатся автоматически.</t>
+          <t>Giper Baza CRDT — real-time sync между клиентами без конфликтов.</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Редактор bog/wysiwyg — отдельный open-source репозиторий https://github.com/b-on-g/wysiwyg.git, лицензия MIT. Построен на $mol (также MIT).</t>
+          <t>https://github.com/b-on-g/wysiwyg.git — MIT лицензия.</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>$bog_wiki_mws_table_live — inline-редактирование ячеек с debounce 1сек → PATCH к MWS Fusion API. Кнопки Add Row (POST), Delete (DELETE), Refresh. Переключение видов (Grid/Gallery) и API-views в тулбаре. Двусторонняя синхронизация.</t>
+          <t>Inline-редактирование ячеек → PATCH к MWS API, debounce 1сек. Add/Delete rows. Grid/Gallery виды.</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Block_comment в каждом блоке wysiwyg. Комментарии привязаны к конкретным блокам контента, хранятся в Giper Baza.</t>
+          <t>Комментарии привязаны к блокам, хранятся в Giper Baza.</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>History panel — просмотр версий страницы. land.fork() для создания снапшотов. Версии хранятся как ссылки в модели Page.Versions.</t>
+          <t>History panel, land.fork() для снапшотов.</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>AI-блок в slash-menu. Генерация контента через LLM API (GitHub Models). Встроен как плагин редактора.</t>
+          <t>AI-блок в slash-menu, генерация через LLM API.</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Graph panel — интерактивная визуализация связей между страницами. Построена на данных wikilinks и backlinks. Навигация по клику на узел графа.</t>
+          <t>Интерактивный граф, навигация по клику на узел.</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>$bog_wysiwyg_plugin_registry — модульная система плагинов. Каждый плагин регистрирует: id, title, on_select(), render(). Новые типы блоков добавляются без изменения ядра редактора. Уже есть: embed, image, code, mws_table, ai.</t>
+          <t>Модульная система плагинов: embed, image, code, mws_table, ai. Новые — без изменения ядра.</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Embed-плагин: вставка YouTube, Vimeo и других iframe-виджетов. Image upload через drag &amp; drop и paste. MWS Table как встроенный виджет. Превью ссылок.</t>
+          <t>Embed (YouTube, Vimeo), image upload (drag &amp; drop, paste), MWS Table inline.</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Нет (Design Kit не применялся). Используются $mol_theme дизайн-токены (светлая/тёмная тема).</t>
+          <t>Не применялся. Используются $mol_theme дизайн-токены.</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Приложение не требует серверной части. Вся логика на клиенте. Giper Baza обеспечивает хранение и синхронизацию. Хостинг — просто статический сайт. Не нужно поднимать БД, писать API, настраивать CI/CD.</t>
+          <t>Вся логика на клиенте. Бэкенд не нужен. Хостинг — статический сайт.</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>End-to-end шифрование по умолчанию в Giper Baza. Даже утечка базы не раскроет данные. Авторизация через криптографические ключи.</t>
+          <t>Giper Baza — E2E шифрование по умолчанию, авторизация через криптоключи.</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Защита периметра не нужна — Giper Baza использует Proof of Work на криптографии для предотвращения спама и DDoS. Не нужен WAF, rate limiting, captcha.</t>
+          <t>Giper Baza Proof of Work — не нужен WAF, rate limiting, captcha.</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Пользователь получает криптографический ключ автоматически при первом открытии сайта. Ни одного клика, ни логина, ни пароля. Профиль сразу доступен.</t>
+          <t>Криптоключ автоматически при первом открытии. Ни логина, ни пароля.</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>CRDT real-time синхронизация без конфликтов</t>
+          <t>Встраивание как Web Component</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Giper Baza CRDT — синхронизация по дельтам между всеми устройствами. Конфликты невозможны на уровне типов данных. Работает через любые ноды-ретрансляторы.</t>
+          <t>WikiLive можно встроить в любой сайт как Web Component.</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>Offline First — полноценная работа без интернета</t>
+          <t>CRDT real-time синхронизация без конфликтов</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Одна строка включает полноценный offline-режим ($mol_offline). Все данные в IndexedDB. Редактирование, создание страниц, навигация — всё работает без сети.</t>
+          <t>CRDT-синхронизация по дельтам, конфликты невозможны на уровне типов данных.</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>Graceful degradation — устойчивость к потере сети</t>
+          <t>Offline First — работа без интернета</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>При потере сети приложение продолжает работать без ошибок. При восстановлении соединения — автоматическая синхронизация всех изменений. Дефолтная фича $mol + Giper Baza.</t>
+          <t>Дефолтное поведение $mol ($mol_offline).</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>Права доступа (owner / editor / viewer)</t>
+          <t>Graceful degradation — устойчивость к потере сети</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -1018,12 +1018,12 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t>Частично</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Визуальная часть готова: UI панели прав, отображение ролей (Owner/Editor/Viewer), скрытие кнопок редактирования для Viewer. Логика Giper Baza land.pass_rank() подключена, но реальное ограничение записи на уровне CRDT пока не проверено в продакшне.</t>
+          <t>Дефолтное поведение $mol + Giper Baza.</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>Адаптивность на все размеры экранов</t>
+          <t>Права доступа (owner / editor / viewer)</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -1043,12 +1043,12 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Частично</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Встроенные механизмы адаптации $mol. Работает на десктопе, планшете, телефоне. Автовиртуализация — рендерятся только видимые элементы.</t>
+          <t>UI готов: панель прав, роли Owner/Editor/Viewer, скрытие кнопок. Логика не проверена в продакшне.</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>Билды под все ОС (Web + Desktop)</t>
+          <t>Адаптивность на все размеры экранов</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Web-приложение работает в любом браузере. Через Tauri возможна сборка нативных десктоп-приложений для macOS, Windows, Linux.</t>
+          <t>Дефолтное поведение $mol.</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>Web Component — приложение как встраиваемый компонент</t>
+          <t>Билды под все ОС (Web + Desktop)</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>Любой $mol-компонент можно зарегистрировать как Web Component через $mol_view_component. WikiLive можно встроить в любой сайт.</t>
+          <t>Web — любой браузер. Desktop — через Tauri (macOS, Windows, Linux).</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Все тексты с @ в view.tree автоматически попадают в файлы перевода. Русский и английский из коробки. Смена языка без перезагрузки. Добавление нового языка — один JSON-файл.</t>
+          <t>Дефолтное поведение $mol. RU + EN из коробки, новый язык = один JSON-файл.</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Граф зависимостей строится автоматически. Пересчитывается и обновляется в DOM только то, что реально изменилось. Нет лишних ре-рендеров. В 3 раза меньше кода чем React + Redux + Router. Дефолтная архитектура $mol.</t>
+          <t>Дефолтная архитектура $mol. Нет Virtual DOM, минимальные обновления DOM.</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>$mol_theme — типизированные дизайн-токены. Переключение светлой/тёмной темы одним кликом. Кастомные темы поддерживаются.</t>
+          <t>Дефолтное поведение $mol. $mol_theme дизайн-токены.</t>
         </is>
       </c>
     </row>

</xml_diff>